<commit_message>
fix: Consolidate database and padron to exact 55 real HikCentral workers (removed unpadded DNI duplicates)
</commit_message>
<xml_diff>
--- a/Padron_Trabajadores_GZG.xlsx
+++ b/Padron_Trabajadores_GZG.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1506,17 +1506,17 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>03208053</t>
+          <t>78197802</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>MORETO BERMEO</t>
+          <t>NEYRA CAMPOS</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>FRANCO</t>
+          <t>YULEISER</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Mantenimiento</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -1538,17 +1538,17 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>78197802</t>
+          <t>47591578</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>NEYRA CAMPOS</t>
+          <t>NINAQUISPE JACOBO</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>YULEISER</t>
+          <t>LUIS MIGUEL</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -1570,17 +1570,17 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>47591578</t>
+          <t>72940900</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>NINAQUISPE JACOBO</t>
+          <t>NOLE LADINES</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>LUIS MIGUEL</t>
+          <t>CARLOS SEBASTIAN</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -1602,7 +1602,7 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>72940900</t>
+          <t>72940901</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>CARLOS SEBASTIAN</t>
+          <t>DIEGO ARMANDO</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -1634,17 +1634,17 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>72940901</t>
+          <t>06616501</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>NOLE LADINES</t>
+          <t>ORDOÑEZ ARTEAGA</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>DIEGO ARMANDO</t>
+          <t>YENKLI VICENTE</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Electricidad</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -1666,17 +1666,17 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>06616501</t>
+          <t>75227437</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>ORDOÑEZ ARTEAGA</t>
+          <t>PRETEL RAMIREZ</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>YENKLI VICENTE</t>
+          <t>LILIANA MORELY</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Electricidad</t>
+          <t>Auxiliar de Seguridad</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -1698,17 +1698,17 @@
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>006616501</t>
+          <t>70088280</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>ORDOÑEZ ARTEAGA</t>
+          <t>RAMIREZ GUERRERO</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>YENKLI VICENTE</t>
+          <t>LUIS FERNANDO</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Electricidad</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -1730,17 +1730,17 @@
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>75227437</t>
+          <t>71060137</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>PRETEL RAMIREZ</t>
+          <t>RAMIREZ LABAN</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>LILIANA MORELY</t>
+          <t>HILDEBRANDO</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Auxiliar de Seguridad</t>
+          <t>Mantenimiento</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -1762,17 +1762,17 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>70088280</t>
+          <t>77386038</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>RAMIREZ GUERRERO</t>
+          <t>RIMARACHIN GARCIA</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO</t>
+          <t>CESAR</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -1794,17 +1794,17 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>71060137</t>
+          <t>71715827</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>RAMIREZ LABAN</t>
+          <t>ROJAS CASTRO</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>HILDEBRANDO</t>
+          <t>ALAN JANDY</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Mantenimiento</t>
+          <t>Maestranza</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -1826,17 +1826,17 @@
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>77386038</t>
+          <t>70639427</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>RIMARACHIN GARCIA</t>
+          <t>RUBIO GUTIERRES</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>CESAR</t>
+          <t>OSBERTO</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -1858,17 +1858,17 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>71715827</t>
+          <t>72500789</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>ROJAS CASTRO</t>
+          <t>SAMBRANO QUISPESIVANA</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>ALAN JANDY</t>
+          <t>ROY IVAN</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Maestranza</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -1890,17 +1890,17 @@
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>70639427</t>
+          <t>70782038</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>RUBIO GUTIERRES</t>
+          <t>SANCHEZ MONTERO</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>OSBERTO</t>
+          <t>JUAN FERNANDO</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -1922,27 +1922,27 @@
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>72500789</t>
+          <t>26696602</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>SAMBRANO QUISPESIVANA</t>
+          <t>SANCHEZ MONTOYA</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>ROY IVAN</t>
+          <t>MANUEL YSIDORO</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Oper&amp;Mtto</t>
+          <t>Jefatura</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Superintendente</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -1954,17 +1954,17 @@
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>70782038</t>
+          <t>44375240</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ MONTERO</t>
+          <t>SANCHEZ PEREZ</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>JUAN FERNANDO</t>
+          <t>EDIN</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Mantenimiento</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -1986,27 +1986,27 @@
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>26696602</t>
+          <t>47721216</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ MONTOYA</t>
+          <t>SANCHEZ RAMIREZ</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>MANUEL YSIDORO</t>
+          <t>PAUL JAIR</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Jefatura</t>
+          <t>Oper&amp;Mtto</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Superintendente</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -2018,17 +2018,17 @@
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>44375240</t>
+          <t>43240513</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ PEREZ</t>
+          <t>SANTOS AGUSTIN</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>EDIN</t>
+          <t>JUAN DIEGO</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Mantenimiento</t>
+          <t>Conductor</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -2050,17 +2050,17 @@
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>47721216</t>
+          <t>41090274</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>SANCHEZ RAMIREZ</t>
+          <t>SILVA CORDOVA</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>PAUL JAIR</t>
+          <t>JUAN PABLO</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2082,17 +2082,17 @@
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>43240513</t>
+          <t>75539351</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>SANTOS AGUSTIN</t>
+          <t>SOLANO GONZALES</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>JUAN DIEGO</t>
+          <t>YERSON</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Conductor</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -2114,17 +2114,17 @@
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>41090274</t>
+          <t>60512609</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>SILVA CORDOVA</t>
+          <t>SUAREZ CAMPOS</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>JUAN PABLO</t>
+          <t>EDERLY</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -2146,27 +2146,27 @@
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>75539351</t>
+          <t>77134790</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>SOLANO GONZALES</t>
+          <t>TOCTO  VALDIVIEZO</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>YERSON</t>
+          <t>CLARI VANESA</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Oper&amp;Mtto</t>
+          <t>Administracion</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -2178,27 +2178,27 @@
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>60512609</t>
+          <t>48455175</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>SUAREZ CAMPOS</t>
+          <t>VASQUEZ PUELLES</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>EDERLY</t>
+          <t>IVAN ANTONIO</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Oper&amp;Mtto</t>
+          <t>Administracion</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -2210,27 +2210,27 @@
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>77134790</t>
+          <t>73485498</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>TOCTO  VALDIVIEZO</t>
+          <t>VEGA CASTILLO</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>CLARI VANESA</t>
+          <t>WILLY LEONARDO</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Administracion</t>
+          <t>Oper&amp;Mtto</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Administrativo</t>
+          <t>Operaciones</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -2242,27 +2242,27 @@
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>48455175</t>
+          <t>41219221</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>VASQUEZ PUELLES</t>
+          <t>VIGO RAFAEL</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>IVAN ANTONIO</t>
+          <t>JOSE ISMAEL</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Administracion</t>
+          <t>Oper&amp;Mtto</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Administrativo</t>
+          <t>Mantenimiento</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -2274,17 +2274,17 @@
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>73485498</t>
+          <t>18861684</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>VEGA CASTILLO</t>
+          <t>ZAMORA CARRASCO</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>WILLY LEONARDO</t>
+          <t>JACOB</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -2294,74 +2294,10 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Electricidad</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>41219221</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>VIGO RAFAEL</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>JOSE ISMAEL</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Oper&amp;Mtto</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Mantenimiento</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>18861684</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>ZAMORA CARRASCO</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>JACOB</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Oper&amp;Mtto</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Electricidad</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>

</xml_diff>

<commit_message>
fix(mobile): persistir base de datos asistencia.db con 35 solicitudes y aprobadores N1/N2 sincronizados, selectores universales CSS para iconos usuario/candado, encabezados proporcionados, estilo rojo elegante en rechazar y popover de clave optimizado
</commit_message>
<xml_diff>
--- a/Padron_Trabajadores_GZG.xlsx
+++ b/Padron_Trabajadores_GZG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GZG Minerales 2026\Desktop\GZG\Sistema_Asistencia_GZG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA9BBBA-BF73-4920-93FA-7A6726A6A656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3BBED4-E7D5-4762-9113-1DB0F8CB46D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trabajadores" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="206">
   <si>
     <t>PADRÓN OFICIAL DE TRABAJADORES Y PERSONAL REGISTRADO - GZG MINERALES</t>
   </si>
@@ -627,6 +627,21 @@
   </si>
   <si>
     <t>Control Total</t>
+  </si>
+  <si>
+    <t>jagreda2026*</t>
+  </si>
+  <si>
+    <t>jalva2026*</t>
+  </si>
+  <si>
+    <t>jdelariva2026*</t>
+  </si>
+  <si>
+    <t>jhuayama2026*</t>
+  </si>
+  <si>
+    <t>msanchez2026*</t>
   </si>
 </sst>
 </file>
@@ -2581,7 +2596,7 @@
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2615,6 +2630,9 @@
       <c r="D2" t="s">
         <v>194</v>
       </c>
+      <c r="E2" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -2629,6 +2647,9 @@
       <c r="D3" t="s">
         <v>193</v>
       </c>
+      <c r="E3" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -2643,6 +2664,9 @@
       <c r="D4" t="s">
         <v>192</v>
       </c>
+      <c r="E4" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -2657,6 +2681,9 @@
       <c r="D5" t="s">
         <v>198</v>
       </c>
+      <c r="E5" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -2670,6 +2697,9 @@
       </c>
       <c r="D6" t="s">
         <v>197</v>
+      </c>
+      <c r="E6" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix(db): actualizar cargo de Javier de la Riva a Jefe y rol JEFE en Padron y DB SQLite
</commit_message>
<xml_diff>
--- a/Padron_Trabajadores_GZG.xlsx
+++ b/Padron_Trabajadores_GZG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GZG Minerales 2026\Desktop\GZG\Sistema_Asistencia_GZG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3BBED4-E7D5-4762-9113-1DB0F8CB46D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053514B6-4E4C-4B99-B30B-0E79AE8C8595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trabajadores" sheetId="1" r:id="rId1"/>
@@ -1081,6 +1081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1147,7 +1148,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -1173,7 +1174,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1199,7 +1200,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1225,7 +1226,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1251,7 +1252,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -1277,7 +1278,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -1303,7 +1304,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -1329,7 +1330,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>37</v>
       </c>
@@ -1355,7 +1356,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
@@ -1381,7 +1382,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -1407,7 +1408,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1433,7 +1434,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -1459,7 +1460,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>52</v>
       </c>
@@ -1485,7 +1486,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>55</v>
       </c>
@@ -1525,7 +1526,7 @@
         <v>21</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>13</v>
@@ -1537,7 +1538,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1563,7 +1564,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>66</v>
       </c>
@@ -1589,7 +1590,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
@@ -1615,7 +1616,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>72</v>
       </c>
@@ -1641,7 +1642,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>75</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>78</v>
       </c>
@@ -1693,7 +1694,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>80</v>
       </c>
@@ -1719,7 +1720,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>83</v>
       </c>
@@ -1745,7 +1746,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>85</v>
       </c>
@@ -1771,7 +1772,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>88</v>
       </c>
@@ -1797,7 +1798,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>91</v>
       </c>
@@ -1823,7 +1824,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>96</v>
       </c>
@@ -1849,7 +1850,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>99</v>
       </c>
@@ -1875,7 +1876,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>102</v>
       </c>
@@ -1901,7 +1902,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>106</v>
       </c>
@@ -1927,7 +1928,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>109</v>
       </c>
@@ -1953,7 +1954,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>112</v>
       </c>
@@ -1979,7 +1980,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>115</v>
       </c>
@@ -2005,7 +2006,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>118</v>
       </c>
@@ -2031,7 +2032,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>120</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>124</v>
       </c>
@@ -2083,7 +2084,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>128</v>
       </c>
@@ -2109,7 +2110,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>131</v>
       </c>
@@ -2135,7 +2136,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>134</v>
       </c>
@@ -2161,7 +2162,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>137</v>
       </c>
@@ -2187,7 +2188,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>140</v>
       </c>
@@ -2213,7 +2214,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>143</v>
       </c>
@@ -2265,7 +2266,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>149</v>
       </c>
@@ -2291,7 +2292,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>153</v>
       </c>
@@ -2317,7 +2318,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>156</v>
       </c>
@@ -2343,7 +2344,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>159</v>
       </c>
@@ -2369,7 +2370,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>163</v>
       </c>
@@ -2395,7 +2396,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>166</v>
       </c>
@@ -2421,7 +2422,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>169</v>
       </c>
@@ -2447,7 +2448,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>172</v>
       </c>
@@ -2473,7 +2474,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>175</v>
       </c>
@@ -2499,7 +2500,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>178</v>
       </c>
@@ -2525,7 +2526,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>181</v>
       </c>
@@ -2551,7 +2552,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>184</v>
       </c>
@@ -2578,7 +2579,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H58" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:H58" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Supervisor"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
padron: retirar a Cristhian Ladines Agurto del padron activo (54 trabajadores)
</commit_message>
<xml_diff>
--- a/Padron_Trabajadores_GZG.xlsx
+++ b/Padron_Trabajadores_GZG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GZG Minerales 2026\Desktop\GZG\Sistema_Asistencia_GZG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053514B6-4E4C-4B99-B30B-0E79AE8C8595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F472FF38-D399-44B2-99E7-C84348C94843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Usuarios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Trabajadores!$A$3:$H$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Trabajadores!$A$3:$H$57</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="204">
   <si>
     <t>PADRÓN OFICIAL DE TRABAJADORES Y PERSONAL REGISTRADO - GZG MINERALES</t>
   </si>
@@ -266,13 +266,7 @@
     <t>MICHAEL JUNIOR</t>
   </si>
   <si>
-    <t>78378144</t>
-  </si>
-  <si>
     <t>LADINES AGURTO</t>
-  </si>
-  <si>
-    <t>CRISTHIAN SINCLAIR</t>
   </si>
   <si>
     <t>62772089</t>
@@ -1081,8 +1075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1142,13 +1135,13 @@
         <v>7</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -1168,13 +1161,13 @@
         <v>13</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1194,13 +1187,13 @@
         <v>13</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1220,13 +1213,13 @@
         <v>13</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1246,13 +1239,13 @@
         <v>13</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -1272,13 +1265,13 @@
         <v>13</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -1298,13 +1291,13 @@
         <v>13</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -1324,13 +1317,13 @@
         <v>13</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>37</v>
       </c>
@@ -1350,13 +1343,13 @@
         <v>13</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
@@ -1376,13 +1369,13 @@
         <v>13</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -1402,13 +1395,13 @@
         <v>13</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1428,13 +1421,13 @@
         <v>13</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -1454,13 +1447,13 @@
         <v>13</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>52</v>
       </c>
@@ -1480,13 +1473,13 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>55</v>
       </c>
@@ -1506,10 +1499,10 @@
         <v>13</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -1532,13 +1525,13 @@
         <v>13</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1558,13 +1551,13 @@
         <v>13</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>66</v>
       </c>
@@ -1584,13 +1577,13 @@
         <v>13</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
@@ -1610,13 +1603,13 @@
         <v>13</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>72</v>
       </c>
@@ -1636,13 +1629,13 @@
         <v>13</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>75</v>
       </c>
@@ -1662,13 +1655,13 @@
         <v>13</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>78</v>
       </c>
@@ -1688,18 +1681,18 @@
         <v>13</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>82</v>
@@ -1708,53 +1701,53 @@
         <v>11</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>11</v>
@@ -1766,177 +1759,177 @@
         <v>13</v>
       </c>
       <c r="G27" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="H27" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="6" t="s">
+      <c r="H28" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="H28" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>94</v>
+        <v>11</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G29" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G29" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E31" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="F33" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>11</v>
@@ -1948,21 +1941,21 @@
         <v>13</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>11</v>
@@ -1974,18 +1967,18 @@
         <v>13</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>117</v>
@@ -2000,203 +1993,203 @@
         <v>13</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>118</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E37" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F37" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H37" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>127</v>
-      </c>
       <c r="F39" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F40" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="F41" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F42" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="F43" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>11</v>
@@ -2208,177 +2201,177 @@
         <v>13</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G45" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H45" s="6" t="s">
         <v>193</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>61</v>
+        <v>150</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G46" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G46" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="H46" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>152</v>
+        <v>36</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G47" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G47" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F49" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G49" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="H49" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>162</v>
-      </c>
       <c r="F50" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G50" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="H50" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G50" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>11</v>
@@ -2390,21 +2383,21 @@
         <v>13</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>11</v>
@@ -2416,176 +2409,144 @@
         <v>13</v>
       </c>
       <c r="G52" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="H52" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="3" t="s">
+      <c r="H53" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="H54" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F53" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G53" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H53" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="F55" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G55" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G55" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="F57" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H58" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Supervisor"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A3:H57" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -2618,10 +2579,10 @@
         <v>4</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2635,10 +2596,10 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2652,10 +2613,10 @@
         <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2669,10 +2630,10 @@
         <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2686,41 +2647,41 @@
         <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>151</v>
-      </c>
       <c r="D6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C7" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E7" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F7" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: Daily attendance & approvals update 9AM
</commit_message>
<xml_diff>
--- a/Padron_Trabajadores_GZG.xlsx
+++ b/Padron_Trabajadores_GZG.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GZG Minerales 2026\Desktop\GZG\Sistema_Asistencia_GZG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F472FF38-D399-44B2-99E7-C84348C94843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3649AD-6EF1-4394-8C7C-57C3F3F91EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Usuarios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Trabajadores!$A$3:$H$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Trabajadores!$A$3:$H$58</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="207">
   <si>
     <t>PADRÓN OFICIAL DE TRABAJADORES Y PERSONAL REGISTRADO - GZG MINERALES</t>
   </si>
@@ -636,6 +636,15 @@
   </si>
   <si>
     <t>msanchez2026*</t>
+  </si>
+  <si>
+    <t>TEJADA VASQUEZ</t>
+  </si>
+  <si>
+    <t>EDGARD STREET</t>
+  </si>
+  <si>
+    <t>73577356</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1084,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H57"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1141,7 +1151,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -1167,7 +1177,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1193,7 +1203,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1219,7 +1229,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1245,7 +1255,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -1271,7 +1281,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -1297,7 +1307,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -1323,7 +1333,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>37</v>
       </c>
@@ -1349,7 +1359,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
@@ -1375,7 +1385,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -1401,7 +1411,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1427,7 +1437,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -1453,7 +1463,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>52</v>
       </c>
@@ -1479,7 +1489,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>55</v>
       </c>
@@ -1505,7 +1515,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>58</v>
       </c>
@@ -1531,7 +1541,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1557,7 +1567,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>66</v>
       </c>
@@ -1583,7 +1593,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
@@ -1609,7 +1619,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>72</v>
       </c>
@@ -1635,7 +1645,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>75</v>
       </c>
@@ -1661,7 +1671,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>78</v>
       </c>
@@ -1687,7 +1697,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>81</v>
       </c>
@@ -1713,7 +1723,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>83</v>
       </c>
@@ -1739,7 +1749,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>86</v>
       </c>
@@ -1765,7 +1775,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>89</v>
       </c>
@@ -1791,7 +1801,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>94</v>
       </c>
@@ -1817,7 +1827,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>97</v>
       </c>
@@ -1843,7 +1853,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>100</v>
       </c>
@@ -1869,7 +1879,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>104</v>
       </c>
@@ -1895,7 +1905,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>107</v>
       </c>
@@ -1921,7 +1931,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>110</v>
       </c>
@@ -1947,7 +1957,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>113</v>
       </c>
@@ -1973,7 +1983,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>116</v>
       </c>
@@ -1999,7 +2009,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>118</v>
       </c>
@@ -2025,7 +2035,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>122</v>
       </c>
@@ -2051,7 +2061,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>126</v>
       </c>
@@ -2077,7 +2087,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>129</v>
       </c>
@@ -2103,7 +2113,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>132</v>
       </c>
@@ -2129,7 +2139,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>135</v>
       </c>
@@ -2155,7 +2165,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>138</v>
       </c>
@@ -2181,7 +2191,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>141</v>
       </c>
@@ -2207,7 +2217,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>144</v>
       </c>
@@ -2233,7 +2243,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>147</v>
       </c>
@@ -2259,7 +2269,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>151</v>
       </c>
@@ -2285,7 +2295,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>154</v>
       </c>
@@ -2311,7 +2321,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>157</v>
       </c>
@@ -2337,7 +2347,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>161</v>
       </c>
@@ -2363,7 +2373,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>164</v>
       </c>
@@ -2389,7 +2399,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>167</v>
       </c>
@@ -2415,7 +2425,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>170</v>
       </c>
@@ -2441,7 +2451,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>173</v>
       </c>
@@ -2467,7 +2477,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>176</v>
       </c>
@@ -2493,7 +2503,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>179</v>
       </c>
@@ -2519,7 +2529,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>182</v>
       </c>
@@ -2545,8 +2555,40 @@
         <v>195</v>
       </c>
     </row>
+    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H57" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:H58" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="TEJADA VASQUEZ"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>